<commit_message>
Added game configurations sheet.
</commit_message>
<xml_diff>
--- a/Documents/AngbandOS.xlsx
+++ b/Documents/AngbandOS.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\AngbandOS\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1385C039-5BDE-458C-BC7D-4D9625EF0815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FE8128-F9D1-43D9-BD80-5150E576E312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30000" yWindow="-90" windowWidth="21600" windowHeight="15990" activeTab="1" xr2:uid="{A03D22A2-317B-4C0C-ACCE-6FB4FF1B36BC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="2" xr2:uid="{A03D22A2-317B-4C0C-ACCE-6FB4FF1B36BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Script Adapters" sheetId="2" r:id="rId2"/>
-    <sheet name="Widgets" sheetId="4" r:id="rId3"/>
-    <sheet name="Functions" sheetId="5" r:id="rId4"/>
+    <sheet name="Game Configurations" sheetId="6" r:id="rId3"/>
+    <sheet name="Widgets" sheetId="4" r:id="rId4"/>
+    <sheet name="Functions" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="176">
   <si>
     <t>IdentifiedResult ExecuteEatOrQuaffScript()</t>
   </si>
@@ -292,6 +292,282 @@
   </si>
   <si>
     <t>GameCommandUniversalScript</t>
+  </si>
+  <si>
+    <t>AbilityScoreScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>Abstracts and Interfaces</t>
+  </si>
+  <si>
+    <t>ActivationGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ActivationNullableReferenceAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>AngbandOS.Core.Interface.Configuration.csproj</t>
+  </si>
+  <si>
+    <t>AnimationGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ArtifactBiasNullableReferenceAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ArtifactBiasWeightedRandomGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>AttackGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>AttributeFilterGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>BoolAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>CauseWoundsMonsterSpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>CharacterClassAbilityGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>CharacterClassSpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ChestTrapCombinationGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ChestTrapGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ColorEnumAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ConditionalGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ConditionalScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ConditionalWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>DamageLearnedKnowledgeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>DateWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>DungeonGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>DungeonGuardianGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>DurationLearnedKnowledgeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ExperienceLearnedKnowledgeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>GameCommandGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>GameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>GameMessageWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>GenderGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>GodGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>HelpGroupGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>IntWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemClassGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemEnhancementGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemEnhancementWeightedRandomGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemFactoryGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemFactoryWeightedRandomGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemFilterGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemFlavorGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ItemIdentificationGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>LabelWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MappedItemEnhancementGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MappedSpellScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MapWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MartialArtsAttackGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MaxRangedWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>MonsterRaceGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>OrAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>OutfitManifestGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>PatronGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>PhysicalAttributeSetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>PluralGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ProjectileGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ProjectileGraphicGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ProjectileMonsterSpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ProjectileScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ProjectileScriptWeightedRandomGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RaceAbilityGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RaceGenderGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RacePowerGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RacialPowerTestGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RangedWeaponBonusGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RangedWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RangeLearnedKnowledgeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RealmCharacterClassGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RealmGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RechargeItemScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>RenderMessageScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ScriptMonsterSpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ShopkeeperGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>StoreCommandGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>StoreFactoryGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>StringNullableReferenceAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>StringWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SumAttributeGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SummonMonsterSpellGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SummonScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SummonWeightedRandomGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SyllableSetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>SymbolGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TalentGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TeleportSelfScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TextWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TileGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TimerScriptGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TimeWidgetGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>TownGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>VaultGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>ViewGameConfiguration.cs</t>
+  </si>
+  <si>
+    <t>WizardCommandGameConfiguration.cs</t>
   </si>
 </sst>
 </file>
@@ -1309,6 +1585,479 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C107AFA-1880-4564-8626-B9C4FC67E6BE}">
+  <dimension ref="A1:A92"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="60.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B935F866-FB85-4D86-88BF-7FBFF2C03DE6}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1317,7 +2066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC030CE4-4F40-4524-9D29-34964B37E929}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>